<commit_message>
updated renderer to edit lines
</commit_message>
<xml_diff>
--- a/he test.xlsx
+++ b/he test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viran\Downloads\indep. project\Graphing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE3659B-5584-4EBD-B01D-8A7138C52016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790E96D2-DC51-4356-9DB6-03DA0B3DF13A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14256" xr2:uid="{085A6C6F-747E-439B-8EF1-4E31859EFEC1}"/>
   </bookViews>
@@ -107,23 +107,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -26884,7 +26868,7 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>